<commit_message>
Motherson PKC Add row in 🏭 Production
</commit_message>
<xml_diff>
--- a/01_Production_Stock_Alert.xlsx
+++ b/01_Production_Stock_Alert.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,10 +469,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -572,6 +570,42 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ALT-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>PRD-NEW-01</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-09-21 16:35</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Assembly Line A</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Motherson PKC Update: 🏭 Production
</commit_message>
<xml_diff>
--- a/01_Production_Stock_Alert.xlsx
+++ b/01_Production_Stock_Alert.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,144 +467,6 @@
           <t>Comments</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>18-01-2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:30</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:30</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:30</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:30</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:30</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:30</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ALT-007</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>PRD-NEW-01</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2026-09-21 16:35</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Assembly Line A</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add product TEST-004 in 🏭 Production
</commit_message>
<xml_diff>
--- a/01_Production_Stock_Alert.xlsx
+++ b/01_Production_Stock_Alert.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA4"/>
+  <dimension ref="A1:AA5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -861,6 +861,61 @@
           <t>In Transit</t>
         </is>
       </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ALT-TEST-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TEST-004</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F5" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L5" t="n">
+        <v>5</v>
+      </c>
+      <c r="M5" t="n">
+        <v>10</v>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-09-23 12:06</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 🏭 Production Department
</commit_message>
<xml_diff>
--- a/01_Production_Stock_Alert.xlsx
+++ b/01_Production_Stock_Alert.xlsx
@@ -556,42 +556,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ALT-003</t>
+          <t>ALT-002</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TEST-003</t>
+          <t>TEST-002</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="F2" t="n">
-        <v>230</v>
+        <v>400</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>🟢 Normal Stock</t>
+          <t>🔴 Shortage</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>🟢 Normal</t>
+          <t>🚨 Critical</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>✅ Normal (Stock OK)</t>
+          <t>🚨 ALERT: 🔴 Shortage (Shortage: 100 units)</t>
         </is>
       </c>
       <c r="K2" t="n">
@@ -608,17 +608,17 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>No Reorder</t>
+          <t>No Reorder Required</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-23 15:09</t>
+          <t>2026-09-23 16:42</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -641,7 +641,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>PO-TEST-003</t>
+          <t>PO-TEST-002</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -659,28 +659,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ALT-002</t>
+          <t>ALT-ALT-005</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TEST-002</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>ALT-005</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
       <c r="E3" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -694,11 +696,11 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>🚨 ALERT: 🔴 Shortage (Shortage: 100.0 units)</t>
+          <t>🚨 ALERT: 🔴 Shortage (Shortage: 99 units)</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L3" t="n">
         <v>5</v>
@@ -707,57 +709,33 @@
         <v>10</v>
       </c>
       <c r="N3" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>No Reorder</t>
+          <t>Reorder Triggered</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-23 15:09</t>
+          <t>2026-09-23 16:42</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Default Supplier</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>PO-TEST-002</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>Road</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>In Transit</t>
-        </is>
-      </c>
+      <c r="AA3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -814,7 +792,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Reorder Required</t>
+          <t>Reorder Triggered</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -824,7 +802,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-23 15:09</t>
+          <t>2026-09-23 16:42</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
@@ -841,7 +819,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ALT-ALT-005</t>
+          <t>ALT-003</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -851,38 +829,36 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ALT-005</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
+          <t>TEST-003</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F5" t="n">
+        <v>230</v>
+      </c>
+      <c r="G5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="n">
-        <v>100</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>99</v>
-      </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>🔴 Shortage</t>
+          <t>🟢 Normal Stock</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>🚨 Critical</t>
+          <t>🟢 Normal</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>🚨 ALERT: 🔴 Shortage (Shortage: 99.0 units)</t>
+          <t>✅ Normal (Stock Optimal)</t>
         </is>
       </c>
       <c r="K5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L5" t="n">
         <v>5</v>
@@ -891,33 +867,57 @@
         <v>10</v>
       </c>
       <c r="N5" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Reorder Required</t>
+          <t>No Reorder Required</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-09-23 15:25</t>
+          <t>2026-09-23 16:42</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Default Supplier</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>PO-TEST-003</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Road</t>
+        </is>
+      </c>
       <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>In Transit</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>✅ Normal (Stock OK)</t>
+          <t>✅ Normal (Stock Optimal)</t>
         </is>
       </c>
       <c r="K6" t="n">
@@ -974,7 +974,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>No Reorder</t>
+          <t>No Reorder Required</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2026-09-23 15:09</t>
+          <t>2026-09-23 16:42</t>
         </is>
       </c>
       <c r="R6" t="inlineStr"/>

</xml_diff>

<commit_message>
Delete product TEST-002 from 🏭 Production Department
</commit_message>
<xml_diff>
--- a/01_Production_Stock_Alert.xlsx
+++ b/01_Production_Stock_Alert.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA6"/>
+  <dimension ref="A1:AA5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,28 +556,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ALT-002</t>
+          <t>ALT-ALT-005</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TEST-002</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>ALT-005</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
       <c r="E2" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -591,11 +593,11 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>🚨 ALERT: 🔴 Shortage (Shortage: 100 units)</t>
+          <t>🚨 ALERT: 🔴 Shortage (Shortage: 99 units)</t>
         </is>
       </c>
       <c r="K2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L2" t="n">
         <v>5</v>
@@ -604,62 +606,38 @@
         <v>10</v>
       </c>
       <c r="N2" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>No Reorder Required</t>
+          <t>Reorder Triggered</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-23 16:43</t>
+          <t>2026-09-23 16:52</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Default Supplier</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>PO-TEST-002</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>Road</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>In Transit</t>
-        </is>
-      </c>
+      <c r="AA2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ALT-ALT-005</t>
+          <t>ALT-TEST-004</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -669,34 +647,32 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ALT-005</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
+          <t>TEST-004</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F3" t="n">
+        <v>11</v>
+      </c>
+      <c r="G3" t="n">
         <v>0</v>
       </c>
-      <c r="E3" t="n">
-        <v>100</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" t="n">
-        <v>99</v>
-      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>🔴 Shortage</t>
+          <t>🟠 Low Stock</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>🚨 Critical</t>
+          <t>🟠 Medium</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>🚨 ALERT: 🔴 Shortage (Shortage: 99 units)</t>
+          <t>⚠️ WARNING: Low Stock Level</t>
         </is>
       </c>
       <c r="K3" t="n">
@@ -718,12 +694,12 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-23 16:43</t>
+          <t>2026-09-23 16:52</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -740,7 +716,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ALT-TEST-004</t>
+          <t>ALT-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -750,36 +726,36 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TEST-004</t>
+          <t>TEST-003</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="F4" t="n">
-        <v>11</v>
+        <v>230</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>🟠 Low Stock</t>
+          <t>🟢 Normal Stock</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>🟠 Medium</t>
+          <t>🟢 Normal</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>⚠️ WARNING: Low Stock Level</t>
+          <t>✅ Normal (Stock Optimal)</t>
         </is>
       </c>
       <c r="K4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L4" t="n">
         <v>5</v>
@@ -788,56 +764,80 @@
         <v>10</v>
       </c>
       <c r="N4" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Reorder Triggered</t>
+          <t>No Reorder Required</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-23 16:43</t>
+          <t>2026-09-23 16:52</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Default Supplier</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>PO-TEST-003</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Road</t>
+        </is>
+      </c>
       <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>In Transit</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ALT-003</t>
+          <t>ALT-001</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TEST-003</t>
+          <t>TEST-001</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>230</v>
+        <v>100</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -876,12 +876,12 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-09-23 16:43</t>
+          <t>2026-09-23 16:52</t>
         </is>
       </c>
       <c r="R5" t="inlineStr"/>
@@ -904,7 +904,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>PO-TEST-003</t>
+          <t>PO-TEST-001</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -914,109 +914,6 @@
       </c>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr">
-        <is>
-          <t>In Transit</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ALT-001</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TEST-001</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="n">
-        <v>100</v>
-      </c>
-      <c r="F6" t="n">
-        <v>100</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>🟢 Normal Stock</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>🟢 Normal</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>✅ Normal (Stock Optimal)</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>7</v>
-      </c>
-      <c r="L6" t="n">
-        <v>5</v>
-      </c>
-      <c r="M6" t="n">
-        <v>10</v>
-      </c>
-      <c r="N6" t="n">
-        <v>45</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>No Reorder Required</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>2026-09-23 16:43</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Default Supplier</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>PO-TEST-001</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>Road</t>
-        </is>
-      </c>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr">
         <is>
           <t>In Transit</t>
         </is>

</xml_diff>

<commit_message>
Delete product ALT-005 from 🏭 Production Department
</commit_message>
<xml_diff>
--- a/01_Production_Stock_Alert.xlsx
+++ b/01_Production_Stock_Alert.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA6"/>
+  <dimension ref="A1:AA5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,7 +556,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ALT-ALT-005</t>
+          <t>ALT-TEST-004</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -566,34 +566,32 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ALT-005</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
+          <t>TEST-004</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F2" t="n">
+        <v>11</v>
+      </c>
+      <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="n">
-        <v>100</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" t="n">
-        <v>99</v>
-      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>🔴 Shortage</t>
+          <t>🟠 Low Stock</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>🚨 Critical</t>
+          <t>🟠 Medium</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>🚨 ALERT: 🔴 Shortage (Shortage: 99 units)</t>
+          <t>⚠️ WARNING: Low Stock Level</t>
         </is>
       </c>
       <c r="K2" t="n">
@@ -615,7 +613,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -637,7 +635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ALT-TEST-004</t>
+          <t>ALT-003</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -647,36 +645,36 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TEST-004</t>
+          <t>TEST-003</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="F3" t="n">
-        <v>11</v>
+        <v>230</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>🟠 Low Stock</t>
+          <t>🟢 Normal Stock</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>🟠 Medium</t>
+          <t>🟢 Normal</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>⚠️ WARNING: Low Stock Level</t>
+          <t>✅ Normal (Stock Optimal)</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L3" t="n">
         <v>5</v>
@@ -685,16 +683,16 @@
         <v>10</v>
       </c>
       <c r="N3" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Reorder Triggered</t>
+          <t>No Reorder Required</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -705,36 +703,60 @@
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Default Supplier</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>PO-TEST-003</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Road</t>
+        </is>
+      </c>
       <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>In Transit</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ALT-003</t>
+          <t>ALT-002</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TEST-003</t>
+          <t>TEST-002</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>230</v>
+        <v>400</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -773,7 +795,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -781,7 +803,11 @@
           <t>2026-09-23 16:53</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Line-A</t>
+        </is>
+      </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr">
@@ -801,7 +827,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>PO-TEST-003</t>
+          <t>PO-TEST-002</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -819,7 +845,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ALT-002</t>
+          <t>ALT-001</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -829,7 +855,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TEST-002</t>
+          <t>TEST-001</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -837,7 +863,7 @@
         <v>100</v>
       </c>
       <c r="F5" t="n">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -876,7 +902,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -884,11 +910,7 @@
           <t>2026-09-23 16:53</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Line-A</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr">
@@ -908,7 +930,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>PO-TEST-002</t>
+          <t>PO-TEST-001</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -918,109 +940,6 @@
       </c>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr">
-        <is>
-          <t>In Transit</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ALT-001</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>TEST-001</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="n">
-        <v>100</v>
-      </c>
-      <c r="F6" t="n">
-        <v>100</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>🟢 Normal Stock</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>🟢 Normal</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>✅ Normal (Stock Optimal)</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>7</v>
-      </c>
-      <c r="L6" t="n">
-        <v>5</v>
-      </c>
-      <c r="M6" t="n">
-        <v>10</v>
-      </c>
-      <c r="N6" t="n">
-        <v>45</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>No Reorder Required</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>2026-09-23 16:53</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Default Supplier</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>PO-TEST-001</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>Road</t>
-        </is>
-      </c>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr">
         <is>
           <t>In Transit</t>
         </is>

</xml_diff>